<commit_message>
ingesta: snapshot 2026-07-20 18:58 UTC
</commit_message>
<xml_diff>
--- a/data_lake/acumulado_tempmax_mes/dt=2026-07-20/Temp-max-julio-26.xlsx
+++ b/data_lake/acumulado_tempmax_mes/dt=2026-07-20/Temp-max-julio-26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C584870-F604-4591-9AC2-81730448EEDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68E3598E-80FA-438C-A021-16AE0125B6CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9478,7 +9478,9 @@
       <c r="V5" s="57">
         <v>30.9</v>
       </c>
-      <c r="W5" s="57"/>
+      <c r="W5" s="57">
+        <v>30.9</v>
+      </c>
       <c r="X5" s="57"/>
       <c r="Y5" s="57"/>
       <c r="Z5" s="57"/>
@@ -9511,11 +9513,11 @@
       </c>
       <c r="AO5" s="23">
         <f>IF(COUNTIF(E5:AI5,"&gt;0")&gt;=15,AVERAGE(E5:AI5),"")</f>
-        <v>31.205555555555559</v>
+        <v>31.189473684210526</v>
       </c>
       <c r="AP5" s="23">
         <f>IF(AN5&gt;0,IFERROR(AO5-AN5,""),"")</f>
-        <v>1.0081837795473305</v>
+        <v>0.99210190820229727</v>
       </c>
     </row>
     <row r="6" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9585,7 +9587,9 @@
       <c r="V6" s="57">
         <v>31.1</v>
       </c>
-      <c r="W6" s="57"/>
+      <c r="W6" s="57">
+        <v>30.8</v>
+      </c>
       <c r="X6" s="57"/>
       <c r="Y6" s="57"/>
       <c r="Z6" s="57"/>
@@ -9600,7 +9604,7 @@
       <c r="AI6" s="57"/>
       <c r="AJ6" s="37">
         <f t="shared" ref="AJ6:AJ48" si="0">+IF(SUM($E6:$AI6)&gt;0,LOOKUP(1000,$E6:$AI6),NA())</f>
-        <v>31.1</v>
+        <v>30.8</v>
       </c>
       <c r="AK6" s="21">
         <f t="shared" ref="AK6:AK48" si="1">+MAX($E6:$AI6)</f>
@@ -9618,11 +9622,11 @@
       </c>
       <c r="AO6" s="23">
         <f t="shared" ref="AO6:AO15" si="3">IF(COUNTIF(E6:AI6,"&gt;0")&gt;=15,AVERAGE(E6:AI6),"")</f>
-        <v>30.655555555555551</v>
+        <v>30.663157894736838</v>
       </c>
       <c r="AP6" s="23">
         <f t="shared" ref="AP6:AP48" si="4">IF(AN6&gt;0,IFERROR(AO6-AN6,""),"")</f>
-        <v>1.2751585332111404E-3</v>
+        <v>8.8774977144971956E-3</v>
       </c>
     </row>
     <row r="7" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9692,7 +9696,9 @@
       <c r="V7" s="57">
         <v>35.799999999999997</v>
       </c>
-      <c r="W7" s="57"/>
+      <c r="W7" s="57">
+        <v>35.9</v>
+      </c>
       <c r="X7" s="57"/>
       <c r="Y7" s="57"/>
       <c r="Z7" s="57"/>
@@ -9707,7 +9713,7 @@
       <c r="AI7" s="57"/>
       <c r="AJ7" s="37">
         <f t="shared" si="0"/>
-        <v>35.799999999999997</v>
+        <v>35.9</v>
       </c>
       <c r="AK7" s="21">
         <f t="shared" si="1"/>
@@ -9725,11 +9731,11 @@
       </c>
       <c r="AO7" s="23">
         <f t="shared" si="3"/>
-        <v>36.18333333333333</v>
+        <v>36.168421052631572</v>
       </c>
       <c r="AP7" s="23">
         <f t="shared" si="4"/>
-        <v>2.8173173257642574</v>
+        <v>2.8024050450624998</v>
       </c>
     </row>
     <row r="8" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9799,7 +9805,9 @@
       <c r="V8" s="57">
         <v>34.1</v>
       </c>
-      <c r="W8" s="57"/>
+      <c r="W8" s="57">
+        <v>32.799999999999997</v>
+      </c>
       <c r="X8" s="57"/>
       <c r="Y8" s="57"/>
       <c r="Z8" s="57"/>
@@ -9814,7 +9822,7 @@
       <c r="AI8" s="57"/>
       <c r="AJ8" s="37">
         <f t="shared" si="0"/>
-        <v>34.1</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="AK8" s="21">
         <f t="shared" si="1"/>
@@ -9832,11 +9840,11 @@
       </c>
       <c r="AO8" s="23">
         <f t="shared" si="3"/>
-        <v>33.466666666666669</v>
+        <v>33.431578947368422</v>
       </c>
       <c r="AP8" s="23">
         <f t="shared" si="4"/>
-        <v>1.2176236559139753</v>
+        <v>1.1825359366157286</v>
       </c>
     </row>
     <row r="9" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -9906,7 +9914,9 @@
       <c r="V9" s="57">
         <v>34.1</v>
       </c>
-      <c r="W9" s="57"/>
+      <c r="W9" s="57">
+        <v>33.200000000000003</v>
+      </c>
       <c r="X9" s="57"/>
       <c r="Y9" s="57"/>
       <c r="Z9" s="57"/>
@@ -9921,7 +9931,7 @@
       <c r="AI9" s="57"/>
       <c r="AJ9" s="37">
         <f t="shared" si="0"/>
-        <v>34.1</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="AK9" s="21">
         <f t="shared" si="1"/>
@@ -9939,11 +9949,11 @@
       </c>
       <c r="AO9" s="23">
         <f t="shared" si="3"/>
-        <v>33.99444444444444</v>
+        <v>33.952631578947368</v>
       </c>
       <c r="AP9" s="23">
         <f t="shared" si="4"/>
-        <v>0.90319830676059354</v>
+        <v>0.86138544126352201</v>
       </c>
     </row>
     <row r="10" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10013,7 +10023,9 @@
       <c r="V10" s="57">
         <v>36.299999999999997</v>
       </c>
-      <c r="W10" s="57"/>
+      <c r="W10" s="57">
+        <v>35.4</v>
+      </c>
       <c r="X10" s="57"/>
       <c r="Y10" s="57"/>
       <c r="Z10" s="57"/>
@@ -10028,7 +10040,7 @@
       <c r="AI10" s="57"/>
       <c r="AJ10" s="37">
         <f t="shared" si="0"/>
-        <v>36.299999999999997</v>
+        <v>35.4</v>
       </c>
       <c r="AK10" s="21">
         <f t="shared" si="1"/>
@@ -10046,11 +10058,11 @@
       </c>
       <c r="AO10" s="23">
         <f t="shared" si="3"/>
-        <v>35.822222222222223</v>
+        <v>35.799999999999997</v>
       </c>
       <c r="AP10" s="23">
         <f t="shared" si="4"/>
-        <v>0.44198399456186621</v>
+        <v>0.41976177233964052</v>
       </c>
     </row>
     <row r="11" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10120,7 +10132,9 @@
       <c r="V11" s="57">
         <v>38.299999999999997</v>
       </c>
-      <c r="W11" s="57"/>
+      <c r="W11" s="57">
+        <v>37</v>
+      </c>
       <c r="X11" s="57"/>
       <c r="Y11" s="57"/>
       <c r="Z11" s="57"/>
@@ -10135,7 +10149,7 @@
       <c r="AI11" s="57"/>
       <c r="AJ11" s="37">
         <f t="shared" si="0"/>
-        <v>38.299999999999997</v>
+        <v>37</v>
       </c>
       <c r="AK11" s="21">
         <f t="shared" si="1"/>
@@ -10153,11 +10167,11 @@
       </c>
       <c r="AO11" s="23">
         <f t="shared" si="3"/>
-        <v>38.349999999999994</v>
+        <v>38.278947368421044</v>
       </c>
       <c r="AP11" s="23">
         <f t="shared" si="4"/>
-        <v>2.812715907151393</v>
+        <v>2.7416632755724422</v>
       </c>
     </row>
     <row r="12" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10227,7 +10241,9 @@
       <c r="V12" s="57">
         <v>35.200000000000003</v>
       </c>
-      <c r="W12" s="57"/>
+      <c r="W12" s="57">
+        <v>32.799999999999997</v>
+      </c>
       <c r="X12" s="57"/>
       <c r="Y12" s="57"/>
       <c r="Z12" s="57"/>
@@ -10242,7 +10258,7 @@
       <c r="AI12" s="57"/>
       <c r="AJ12" s="37">
         <f t="shared" si="0"/>
-        <v>35.200000000000003</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="AK12" s="21">
         <f t="shared" si="1"/>
@@ -10260,11 +10276,11 @@
       </c>
       <c r="AO12" s="23">
         <f t="shared" si="3"/>
-        <v>35.088888888888889</v>
+        <v>34.968421052631577</v>
       </c>
       <c r="AP12" s="23">
         <f t="shared" si="4"/>
-        <v>2.9002647427151516</v>
+        <v>2.7797969064578396</v>
       </c>
     </row>
     <row r="13" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10334,7 +10350,9 @@
       <c r="V13" s="57">
         <v>36.799999999999997</v>
       </c>
-      <c r="W13" s="57"/>
+      <c r="W13" s="57">
+        <v>34.6</v>
+      </c>
       <c r="X13" s="57"/>
       <c r="Y13" s="57"/>
       <c r="Z13" s="57"/>
@@ -10349,7 +10367,7 @@
       <c r="AI13" s="57"/>
       <c r="AJ13" s="37">
         <f t="shared" si="0"/>
-        <v>36.799999999999997</v>
+        <v>34.6</v>
       </c>
       <c r="AK13" s="21">
         <f t="shared" si="1"/>
@@ -10367,11 +10385,11 @@
       </c>
       <c r="AO13" s="23">
         <f t="shared" si="3"/>
-        <v>36.299999999999997</v>
+        <v>36.210526315789473</v>
       </c>
       <c r="AP13" s="23">
         <f t="shared" si="4"/>
-        <v>2.9182078853046605</v>
+        <v>2.8287342010941359</v>
       </c>
     </row>
     <row r="14" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10441,7 +10459,9 @@
       <c r="V14" s="57">
         <v>36.700000000000003</v>
       </c>
-      <c r="W14" s="57"/>
+      <c r="W14" s="57">
+        <v>33</v>
+      </c>
       <c r="X14" s="57"/>
       <c r="Y14" s="57"/>
       <c r="Z14" s="57"/>
@@ -10456,7 +10476,7 @@
       <c r="AI14" s="57"/>
       <c r="AJ14" s="37">
         <f t="shared" si="0"/>
-        <v>36.700000000000003</v>
+        <v>33</v>
       </c>
       <c r="AK14" s="21">
         <f t="shared" si="1"/>
@@ -10474,11 +10494,11 @@
       </c>
       <c r="AO14" s="23">
         <f t="shared" si="3"/>
-        <v>35.383333333333333</v>
+        <v>35.257894736842104</v>
       </c>
       <c r="AP14" s="23">
         <f t="shared" si="4"/>
-        <v>2.1583967341191013</v>
+        <v>2.0329581376278725</v>
       </c>
     </row>
     <row r="15" spans="1:46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10548,7 +10568,9 @@
       <c r="V15" s="57">
         <v>33.1</v>
       </c>
-      <c r="W15" s="57"/>
+      <c r="W15" s="57">
+        <v>29.5</v>
+      </c>
       <c r="X15" s="57"/>
       <c r="Y15" s="57"/>
       <c r="Z15" s="57"/>
@@ -10563,7 +10585,7 @@
       <c r="AI15" s="57"/>
       <c r="AJ15" s="37">
         <f t="shared" si="0"/>
-        <v>33.1</v>
+        <v>29.5</v>
       </c>
       <c r="AK15" s="21">
         <f t="shared" si="1"/>
@@ -10581,11 +10603,11 @@
       </c>
       <c r="AO15" s="23">
         <f t="shared" si="3"/>
-        <v>31.966666666666665</v>
+        <v>31.836842105263155</v>
       </c>
       <c r="AP15" s="23">
         <f t="shared" si="4"/>
-        <v>0.23132921058671485</v>
+        <v>0.10150464918320523</v>
       </c>
     </row>
     <row r="16" spans="1:46" s="2" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -10704,7 +10726,9 @@
       <c r="V17" s="57">
         <v>35.799999999999997</v>
       </c>
-      <c r="W17" s="57"/>
+      <c r="W17" s="57">
+        <v>32.4</v>
+      </c>
       <c r="X17" s="57"/>
       <c r="Y17" s="57"/>
       <c r="Z17" s="57"/>
@@ -10719,7 +10743,7 @@
       <c r="AI17" s="57"/>
       <c r="AJ17" s="37">
         <f t="shared" si="0"/>
-        <v>35.799999999999997</v>
+        <v>32.4</v>
       </c>
       <c r="AK17" s="21">
         <f t="shared" si="1"/>
@@ -10737,11 +10761,11 @@
       </c>
       <c r="AO17" s="23">
         <f>IF(COUNTIF(E17:AI17,"&gt;0")&gt;=15,AVERAGE(E17:AI17),"")</f>
-        <v>34.74444444444444</v>
+        <v>34.621052631578941</v>
       </c>
       <c r="AP17" s="23">
         <f>IF(AN17&gt;0,IFERROR(AO17-AN17,""),"")</f>
-        <v>2.0704622419972836</v>
+        <v>1.9470704291317844</v>
       </c>
     </row>
     <row r="18" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10811,7 +10835,9 @@
       <c r="V18" s="57">
         <v>27.6</v>
       </c>
-      <c r="W18" s="57"/>
+      <c r="W18" s="57">
+        <v>26.9</v>
+      </c>
       <c r="X18" s="57"/>
       <c r="Y18" s="57"/>
       <c r="Z18" s="57"/>
@@ -10826,7 +10852,7 @@
       <c r="AI18" s="57"/>
       <c r="AJ18" s="37">
         <f t="shared" si="0"/>
-        <v>27.6</v>
+        <v>26.9</v>
       </c>
       <c r="AK18" s="21">
         <f t="shared" si="1"/>
@@ -10844,11 +10870,11 @@
       </c>
       <c r="AO18" s="23">
         <f t="shared" ref="AO18:AO33" si="5">IF(COUNTIF(E18:AI18,"&gt;0")&gt;=15,AVERAGE(E18:AI18),"")</f>
-        <v>28.205555555555563</v>
+        <v>28.136842105263167</v>
       </c>
       <c r="AP18" s="23">
         <f t="shared" si="4"/>
-        <v>2.1456847015986931</v>
+        <v>2.076971251306297</v>
       </c>
     </row>
     <row r="19" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -10918,7 +10944,9 @@
       <c r="V19" s="57">
         <v>32.299999999999997</v>
       </c>
-      <c r="W19" s="57"/>
+      <c r="W19" s="57">
+        <v>34.1</v>
+      </c>
       <c r="X19" s="57"/>
       <c r="Y19" s="57"/>
       <c r="Z19" s="57"/>
@@ -10933,7 +10961,7 @@
       <c r="AI19" s="57"/>
       <c r="AJ19" s="37">
         <f t="shared" si="0"/>
-        <v>32.299999999999997</v>
+        <v>34.1</v>
       </c>
       <c r="AK19" s="21">
         <f t="shared" si="1"/>
@@ -10951,11 +10979,11 @@
       </c>
       <c r="AO19" s="23">
         <f t="shared" si="5"/>
-        <v>33.766666666666666</v>
+        <v>33.784210526315789</v>
       </c>
       <c r="AP19" s="23">
         <f t="shared" si="4"/>
-        <v>0.51570426399702285</v>
+        <v>0.53324812364614615</v>
       </c>
     </row>
     <row r="20" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11025,7 +11053,9 @@
       <c r="V20" s="57">
         <v>31.8</v>
       </c>
-      <c r="W20" s="57"/>
+      <c r="W20" s="57">
+        <v>28.6</v>
+      </c>
       <c r="X20" s="57"/>
       <c r="Y20" s="57"/>
       <c r="Z20" s="57"/>
@@ -11040,7 +11070,7 @@
       <c r="AI20" s="57"/>
       <c r="AJ20" s="37">
         <f t="shared" si="0"/>
-        <v>31.8</v>
+        <v>28.6</v>
       </c>
       <c r="AK20" s="21">
         <f t="shared" si="1"/>
@@ -11058,11 +11088,11 @@
       </c>
       <c r="AO20" s="23">
         <f t="shared" si="5"/>
-        <v>30.677777777777781</v>
+        <v>30.568421052631582</v>
       </c>
       <c r="AP20" s="23">
         <f t="shared" si="4"/>
-        <v>2.0369731800766324</v>
+        <v>1.9276164549304333</v>
       </c>
     </row>
     <row r="21" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11132,7 +11162,9 @@
       <c r="V21" s="57">
         <v>24.9</v>
       </c>
-      <c r="W21" s="57"/>
+      <c r="W21" s="57">
+        <v>23.7</v>
+      </c>
       <c r="X21" s="57"/>
       <c r="Y21" s="57"/>
       <c r="Z21" s="57"/>
@@ -11147,7 +11179,7 @@
       <c r="AI21" s="57"/>
       <c r="AJ21" s="37">
         <f t="shared" si="0"/>
-        <v>24.9</v>
+        <v>23.7</v>
       </c>
       <c r="AK21" s="21">
         <f t="shared" si="1"/>
@@ -11165,11 +11197,11 @@
       </c>
       <c r="AO21" s="23">
         <f t="shared" si="5"/>
-        <v>24.455555555555552</v>
+        <v>24.415789473684207</v>
       </c>
       <c r="AP21" s="23">
         <f t="shared" si="4"/>
-        <v>1.8460524039055812</v>
+        <v>1.8062863220342358</v>
       </c>
     </row>
     <row r="22" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11307,7 +11339,9 @@
       <c r="V23" s="57">
         <v>28.5</v>
       </c>
-      <c r="W23" s="57"/>
+      <c r="W23" s="57">
+        <v>24</v>
+      </c>
       <c r="X23" s="57"/>
       <c r="Y23" s="57"/>
       <c r="Z23" s="57"/>
@@ -11322,7 +11356,7 @@
       <c r="AI23" s="57"/>
       <c r="AJ23" s="37">
         <f t="shared" si="0"/>
-        <v>28.5</v>
+        <v>24</v>
       </c>
       <c r="AK23" s="21">
         <f t="shared" si="1"/>
@@ -11340,11 +11374,11 @@
       </c>
       <c r="AO23" s="23">
         <f t="shared" si="5"/>
-        <v>28.983333333333334</v>
+        <v>28.721052631578949</v>
       </c>
       <c r="AP23" s="23">
         <f t="shared" si="4"/>
-        <v>2.1149462365591347</v>
+        <v>1.8526655348047498</v>
       </c>
     </row>
     <row r="24" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11414,7 +11448,9 @@
       <c r="V24" s="57">
         <v>29.6</v>
       </c>
-      <c r="W24" s="57"/>
+      <c r="W24" s="57">
+        <v>24.9</v>
+      </c>
       <c r="X24" s="57"/>
       <c r="Y24" s="57"/>
       <c r="Z24" s="57"/>
@@ -11429,7 +11465,7 @@
       <c r="AI24" s="57"/>
       <c r="AJ24" s="37">
         <f t="shared" si="0"/>
-        <v>29.6</v>
+        <v>24.9</v>
       </c>
       <c r="AK24" s="21">
         <f t="shared" si="1"/>
@@ -11447,11 +11483,11 @@
       </c>
       <c r="AO24" s="23">
         <f t="shared" si="5"/>
-        <v>30.061111111111114</v>
+        <v>29.789473684210527</v>
       </c>
       <c r="AP24" s="23">
         <f t="shared" si="4"/>
-        <v>1.809286994367632</v>
+        <v>1.5376495674670458</v>
       </c>
     </row>
     <row r="25" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11521,7 +11557,9 @@
       <c r="V25" s="57">
         <v>31.1</v>
       </c>
-      <c r="W25" s="57"/>
+      <c r="W25" s="57">
+        <v>31.2</v>
+      </c>
       <c r="X25" s="57"/>
       <c r="Y25" s="57"/>
       <c r="Z25" s="57"/>
@@ -11536,7 +11574,7 @@
       <c r="AI25" s="57"/>
       <c r="AJ25" s="37">
         <f t="shared" si="0"/>
-        <v>31.1</v>
+        <v>31.2</v>
       </c>
       <c r="AK25" s="21">
         <f t="shared" si="1"/>
@@ -11554,11 +11592,11 @@
       </c>
       <c r="AO25" s="23">
         <f t="shared" si="5"/>
-        <v>32.305555555555564</v>
+        <v>32.247368421052641</v>
       </c>
       <c r="AP25" s="23">
         <f t="shared" si="4"/>
-        <v>1.9296901623344951</v>
+        <v>1.8715030278315723</v>
       </c>
     </row>
     <row r="26" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11628,7 +11666,9 @@
       <c r="V26" s="57">
         <v>20.6</v>
       </c>
-      <c r="W26" s="57"/>
+      <c r="W26" s="57">
+        <v>19.3</v>
+      </c>
       <c r="X26" s="57"/>
       <c r="Y26" s="57"/>
       <c r="Z26" s="57"/>
@@ -11643,7 +11683,7 @@
       <c r="AI26" s="57"/>
       <c r="AJ26" s="37">
         <f t="shared" si="0"/>
-        <v>20.6</v>
+        <v>19.3</v>
       </c>
       <c r="AK26" s="21">
         <f t="shared" si="1"/>
@@ -11661,11 +11701,11 @@
       </c>
       <c r="AO26" s="23">
         <f t="shared" si="5"/>
-        <v>19.683333333333337</v>
+        <v>19.663157894736845</v>
       </c>
       <c r="AP26" s="23">
         <f t="shared" si="4"/>
-        <v>1.1404617258899776</v>
+        <v>1.1202862872934851</v>
       </c>
     </row>
     <row r="27" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11735,7 +11775,9 @@
       <c r="V27" s="57">
         <v>21.8</v>
       </c>
-      <c r="W27" s="57"/>
+      <c r="W27" s="57">
+        <v>20.399999999999999</v>
+      </c>
       <c r="X27" s="57"/>
       <c r="Y27" s="57"/>
       <c r="Z27" s="57"/>
@@ -11750,7 +11792,7 @@
       <c r="AI27" s="57"/>
       <c r="AJ27" s="37">
         <f t="shared" si="0"/>
-        <v>21.8</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="AK27" s="21">
         <f t="shared" si="1"/>
@@ -11768,11 +11810,11 @@
       </c>
       <c r="AO27" s="23">
         <f t="shared" si="5"/>
-        <v>18.505555555555553</v>
+        <v>18.605263157894733</v>
       </c>
       <c r="AP27" s="23">
         <f t="shared" si="4"/>
-        <v>1.823505011447164</v>
+        <v>1.9232126137863439</v>
       </c>
     </row>
     <row r="28" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -11842,7 +11884,9 @@
       <c r="V28" s="57">
         <v>30.5</v>
       </c>
-      <c r="W28" s="57"/>
+      <c r="W28" s="57">
+        <v>29.1</v>
+      </c>
       <c r="X28" s="57"/>
       <c r="Y28" s="57"/>
       <c r="Z28" s="57"/>
@@ -11857,7 +11901,7 @@
       <c r="AI28" s="57"/>
       <c r="AJ28" s="37">
         <f t="shared" si="0"/>
-        <v>30.5</v>
+        <v>29.1</v>
       </c>
       <c r="AK28" s="21">
         <f t="shared" si="1"/>
@@ -11875,11 +11919,11 @@
       </c>
       <c r="AO28" s="23">
         <f t="shared" si="5"/>
-        <v>32.12777777777778</v>
+        <v>31.968421052631584</v>
       </c>
       <c r="AP28" s="23">
         <f t="shared" si="4"/>
-        <v>1.5993251761216207</v>
+        <v>1.4399684509754245</v>
       </c>
     </row>
     <row r="29" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12015,7 +12059,9 @@
       <c r="V30" s="57">
         <v>31.8</v>
       </c>
-      <c r="W30" s="57"/>
+      <c r="W30" s="57">
+        <v>33.200000000000003</v>
+      </c>
       <c r="X30" s="57"/>
       <c r="Y30" s="57"/>
       <c r="Z30" s="57"/>
@@ -12030,7 +12076,7 @@
       <c r="AI30" s="57"/>
       <c r="AJ30" s="37">
         <f t="shared" si="0"/>
-        <v>31.8</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="AK30" s="21">
         <f t="shared" si="1"/>
@@ -12048,11 +12094,11 @@
       </c>
       <c r="AO30" s="23">
         <f t="shared" si="5"/>
-        <v>34.572222222222223</v>
+        <v>34.500000000000007</v>
       </c>
       <c r="AP30" s="23">
         <f t="shared" si="4"/>
-        <v>0.82997132616487335</v>
+        <v>0.7577491039426576</v>
       </c>
     </row>
     <row r="31" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12122,7 +12168,9 @@
       <c r="V31" s="57">
         <v>27.4</v>
       </c>
-      <c r="W31" s="57"/>
+      <c r="W31" s="57">
+        <v>23.8</v>
+      </c>
       <c r="X31" s="57"/>
       <c r="Y31" s="57"/>
       <c r="Z31" s="57"/>
@@ -12137,7 +12185,7 @@
       <c r="AI31" s="57"/>
       <c r="AJ31" s="37">
         <f t="shared" si="0"/>
-        <v>27.4</v>
+        <v>23.8</v>
       </c>
       <c r="AK31" s="21">
         <f t="shared" si="1"/>
@@ -12155,11 +12203,11 @@
       </c>
       <c r="AO31" s="23">
         <f t="shared" si="5"/>
-        <v>27.75</v>
+        <v>27.542105263157893</v>
       </c>
       <c r="AP31" s="23">
         <f t="shared" si="4"/>
-        <v>2.3625751628793807</v>
+        <v>2.1546804260372738</v>
       </c>
     </row>
     <row r="32" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12229,7 +12277,9 @@
       <c r="V32" s="57">
         <v>18.2</v>
       </c>
-      <c r="W32" s="57"/>
+      <c r="W32" s="57">
+        <v>17.600000000000001</v>
+      </c>
       <c r="X32" s="57"/>
       <c r="Y32" s="57"/>
       <c r="Z32" s="57"/>
@@ -12244,7 +12294,7 @@
       <c r="AI32" s="57"/>
       <c r="AJ32" s="37">
         <f t="shared" si="0"/>
-        <v>18.2</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="AK32" s="21">
         <f t="shared" si="1"/>
@@ -12262,11 +12312,11 @@
       </c>
       <c r="AO32" s="23">
         <f t="shared" si="5"/>
-        <v>17.87777777777778</v>
+        <v>17.863157894736844</v>
       </c>
       <c r="AP32" s="23">
         <f t="shared" si="4"/>
-        <v>1.5482400045165292</v>
+        <v>1.5336201214755931</v>
       </c>
     </row>
     <row r="33" spans="1:47" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -12336,7 +12386,9 @@
       <c r="V33" s="57">
         <v>16</v>
       </c>
-      <c r="W33" s="57"/>
+      <c r="W33" s="57">
+        <v>16.2</v>
+      </c>
       <c r="X33" s="57"/>
       <c r="Y33" s="57"/>
       <c r="Z33" s="57"/>
@@ -12351,7 +12403,7 @@
       <c r="AI33" s="57"/>
       <c r="AJ33" s="37">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>16.2</v>
       </c>
       <c r="AK33" s="21">
         <f t="shared" si="1"/>
@@ -12369,11 +12421,11 @@
       </c>
       <c r="AO33" s="23">
         <f t="shared" si="5"/>
-        <v>15.638888888888889</v>
+        <v>15.668421052631578</v>
       </c>
       <c r="AP33" s="23">
         <f t="shared" si="4"/>
-        <v>0.8942763564454399</v>
+        <v>0.92380852018812831</v>
       </c>
       <c r="AT33" s="15"/>
     </row>
@@ -12495,7 +12547,9 @@
       <c r="V35" s="57">
         <v>32.4</v>
       </c>
-      <c r="W35" s="57"/>
+      <c r="W35" s="57">
+        <v>28</v>
+      </c>
       <c r="X35" s="57"/>
       <c r="Y35" s="57"/>
       <c r="Z35" s="57"/>
@@ -12510,7 +12564,7 @@
       <c r="AI35" s="57"/>
       <c r="AJ35" s="37">
         <f t="shared" si="0"/>
-        <v>32.4</v>
+        <v>28</v>
       </c>
       <c r="AK35" s="21">
         <f t="shared" si="1"/>
@@ -12528,11 +12582,11 @@
       </c>
       <c r="AO35" s="23">
         <f>IF(COUNTIF(E35:AI35,"&gt;0")&gt;=15,AVERAGE(E35:AI35),"")</f>
-        <v>32.24444444444444</v>
+        <v>32.021052631578939</v>
       </c>
       <c r="AP35" s="23">
         <f t="shared" si="4"/>
-        <v>1.1717485919098785</v>
+        <v>0.94835677904437787</v>
       </c>
       <c r="AT35" s="15"/>
     </row>
@@ -12723,7 +12777,9 @@
       <c r="V38" s="57">
         <v>31.8</v>
       </c>
-      <c r="W38" s="57"/>
+      <c r="W38" s="57">
+        <v>31.5</v>
+      </c>
       <c r="X38" s="57"/>
       <c r="Y38" s="57"/>
       <c r="Z38" s="57"/>
@@ -12738,7 +12794,7 @@
       <c r="AI38" s="57"/>
       <c r="AJ38" s="37">
         <f t="shared" si="0"/>
-        <v>31.8</v>
+        <v>31.5</v>
       </c>
       <c r="AK38" s="21">
         <f t="shared" si="1"/>
@@ -12756,11 +12812,11 @@
       </c>
       <c r="AO38" s="23">
         <f>IF(COUNTIF(E38:AI38,"&gt;0")&gt;=15,AVERAGE(E38:AI38),"")</f>
-        <v>30.166666666666661</v>
+        <v>30.23684210526315</v>
       </c>
       <c r="AP38" s="23">
         <f t="shared" si="4"/>
-        <v>0.13764044327407987</v>
+        <v>0.20781588187056954</v>
       </c>
       <c r="AT38" s="15"/>
     </row>
@@ -12831,7 +12887,9 @@
       <c r="V39" s="57">
         <v>30.2</v>
       </c>
-      <c r="W39" s="57"/>
+      <c r="W39" s="57">
+        <v>29</v>
+      </c>
       <c r="X39" s="57"/>
       <c r="Y39" s="57"/>
       <c r="Z39" s="57"/>
@@ -12846,7 +12904,7 @@
       <c r="AI39" s="57"/>
       <c r="AJ39" s="37">
         <f t="shared" si="0"/>
-        <v>30.2</v>
+        <v>29</v>
       </c>
       <c r="AK39" s="21">
         <f t="shared" si="1"/>
@@ -12864,11 +12922,11 @@
       </c>
       <c r="AO39" s="23">
         <f t="shared" ref="AO39:AO48" si="7">IF(COUNTIF(E39:AI39,"&gt;0")&gt;=15,AVERAGE(E39:AI39),"")</f>
-        <v>31.333333333333332</v>
+        <v>31.210526315789473</v>
       </c>
       <c r="AP39" s="23">
         <f t="shared" si="4"/>
-        <v>0.49020022246941153</v>
+        <v>0.36739320492555194</v>
       </c>
       <c r="AT39" s="15"/>
     </row>
@@ -12939,7 +12997,9 @@
       <c r="V40" s="57">
         <v>29.2</v>
       </c>
-      <c r="W40" s="57"/>
+      <c r="W40" s="57">
+        <v>30.2</v>
+      </c>
       <c r="X40" s="57"/>
       <c r="Y40" s="57"/>
       <c r="Z40" s="57"/>
@@ -12954,7 +13014,7 @@
       <c r="AI40" s="57"/>
       <c r="AJ40" s="37">
         <f t="shared" si="0"/>
-        <v>29.2</v>
+        <v>30.2</v>
       </c>
       <c r="AK40" s="21">
         <f t="shared" si="1"/>
@@ -12972,11 +13032,11 @@
       </c>
       <c r="AO40" s="23">
         <f t="shared" si="7"/>
-        <v>29.433333333333337</v>
+        <v>29.473684210526322</v>
       </c>
       <c r="AP40" s="23">
         <f t="shared" si="4"/>
-        <v>0.48578494623655644</v>
+        <v>0.52613582342954146</v>
       </c>
       <c r="AT40" s="15"/>
     </row>
@@ -13047,7 +13107,9 @@
       <c r="V41" s="57">
         <v>29.6</v>
       </c>
-      <c r="W41" s="57"/>
+      <c r="W41" s="57">
+        <v>29.2</v>
+      </c>
       <c r="X41" s="57"/>
       <c r="Y41" s="57"/>
       <c r="Z41" s="57"/>
@@ -13062,7 +13124,7 @@
       <c r="AI41" s="57"/>
       <c r="AJ41" s="37">
         <f t="shared" si="0"/>
-        <v>29.6</v>
+        <v>29.2</v>
       </c>
       <c r="AK41" s="21">
         <f t="shared" si="1"/>
@@ -13080,11 +13142,11 @@
       </c>
       <c r="AO41" s="23">
         <f t="shared" si="7"/>
-        <v>30.455555555555559</v>
+        <v>30.389473684210532</v>
       </c>
       <c r="AP41" s="23">
         <f t="shared" si="4"/>
-        <v>1.0892473118279682</v>
+        <v>1.0231654404829413</v>
       </c>
       <c r="AT41" s="15"/>
     </row>
@@ -13216,7 +13278,9 @@
       <c r="V43" s="57">
         <v>31.2</v>
       </c>
-      <c r="W43" s="57"/>
+      <c r="W43" s="57">
+        <v>26.6</v>
+      </c>
       <c r="X43" s="57"/>
       <c r="Y43" s="57"/>
       <c r="Z43" s="57"/>
@@ -13231,7 +13295,7 @@
       <c r="AI43" s="57"/>
       <c r="AJ43" s="37">
         <f t="shared" si="0"/>
-        <v>31.2</v>
+        <v>26.6</v>
       </c>
       <c r="AK43" s="21">
         <f t="shared" si="1"/>
@@ -13249,11 +13313,11 @@
       </c>
       <c r="AO43" s="23">
         <f t="shared" si="7"/>
-        <v>30.973333333333333</v>
+        <v>30.7</v>
       </c>
       <c r="AP43" s="23">
         <f t="shared" si="4"/>
-        <v>0.91227150537634216</v>
+        <v>0.63893817204300873</v>
       </c>
       <c r="AT43" s="15"/>
     </row>
@@ -13322,7 +13386,9 @@
       <c r="V44" s="29">
         <v>31.1</v>
       </c>
-      <c r="W44" s="29"/>
+      <c r="W44" s="29">
+        <v>30.3</v>
+      </c>
       <c r="X44" s="29"/>
       <c r="Y44" s="29"/>
       <c r="Z44" s="29"/>
@@ -13337,7 +13403,7 @@
       <c r="AI44" s="57"/>
       <c r="AJ44" s="37">
         <f t="shared" si="0"/>
-        <v>31.1</v>
+        <v>30.3</v>
       </c>
       <c r="AK44" s="21">
         <f t="shared" si="1"/>
@@ -13355,11 +13421,11 @@
       </c>
       <c r="AO44" s="23">
         <f t="shared" si="7"/>
-        <v>31.217647058823527</v>
+        <v>31.166666666666661</v>
       </c>
       <c r="AP44" s="23">
         <f t="shared" si="4"/>
-        <v>2.1744598534630661</v>
+        <v>2.1234794613062</v>
       </c>
       <c r="AT44" s="15"/>
     </row>
@@ -13430,7 +13496,9 @@
       <c r="V45" s="57">
         <v>29.8</v>
       </c>
-      <c r="W45" s="57"/>
+      <c r="W45" s="57">
+        <v>27.2</v>
+      </c>
       <c r="X45" s="57"/>
       <c r="Y45" s="57"/>
       <c r="Z45" s="57"/>
@@ -13445,7 +13513,7 @@
       <c r="AI45" s="57"/>
       <c r="AJ45" s="37">
         <f t="shared" si="0"/>
-        <v>29.8</v>
+        <v>27.2</v>
       </c>
       <c r="AK45" s="21">
         <f t="shared" si="1"/>
@@ -13463,11 +13531,11 @@
       </c>
       <c r="AO45" s="23">
         <f t="shared" si="7"/>
-        <v>30.411111111111115</v>
+        <v>30.242105263157903</v>
       </c>
       <c r="AP45" s="23">
         <f t="shared" si="4"/>
-        <v>0.86529471823228477</v>
+        <v>0.69628887027907282</v>
       </c>
       <c r="AT45" s="15"/>
     </row>
@@ -13677,7 +13745,9 @@
       <c r="V48" s="57">
         <v>32.9</v>
       </c>
-      <c r="W48" s="57"/>
+      <c r="W48" s="57">
+        <v>32.9</v>
+      </c>
       <c r="X48" s="57"/>
       <c r="Y48" s="57"/>
       <c r="Z48" s="57"/>
@@ -13710,11 +13780,11 @@
       </c>
       <c r="AO48" s="23">
         <f t="shared" si="7"/>
-        <v>30.261111111111113</v>
+        <v>30.400000000000002</v>
       </c>
       <c r="AP48" s="23">
         <f t="shared" si="4"/>
-        <v>-8.1421744324966738E-2</v>
+        <v>5.7467144563922545E-2</v>
       </c>
     </row>
     <row r="49" spans="5:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -26613,6 +26683,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
     <mergeCell ref="O1:O2"/>
@@ -26622,12 +26698,6 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="L1:L2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:O13 D15:O31 D33:O34 D36:O46">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>